<commit_message>
Add May exchange rates, deduplicate April
</commit_message>
<xml_diff>
--- a/data/exchange_rates/exchange_rate.xlsx
+++ b/data/exchange_rates/exchange_rate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\skynet\kpi_dash\data\exchange_rates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EBF267-B126-4BA0-BB9A-C71D39DF509D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CA5D2E-B2AE-40FF-B3AC-2D53AE98E8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-708" windowWidth="23256" windowHeight="13896" xr2:uid="{6A86D2FA-C3E4-4C0B-B37D-CE9A93AF40E3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6A86D2FA-C3E4-4C0B-B37D-CE9A93AF40E3}"/>
   </bookViews>
   <sheets>
     <sheet name="exchange_rate" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="16">
   <si>
     <t>month</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
   </si>
 </sst>
 </file>
@@ -1164,7 +1167,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -1181,7 +1184,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>8</v>
@@ -1198,7 +1201,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>

</xml_diff>